<commit_message>
Codigo inicial de Cenco
INSERT

a
""
:wq

:wq
:q!
</commit_message>
<xml_diff>
--- a/app/Archivos/Template/Template_HRC_olimpica.xlsx
+++ b/app/Archivos/Template/Template_HRC_olimpica.xlsx
@@ -7115,10 +7115,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{89db4e91-bad5-4fd0-9ca4-c06485916e3a}" enabled="1" method="Standard" siteId="{f66fae02-5d36-495b-bfe0-78a6ff9f8e6e}" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>